<commit_message>
Add academic statistics (95% CI, p, OR) to N=400 reports and admin panel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/reports/n400/Anketa_Tahlili_N400.xlsx
+++ b/public/reports/n400/Anketa_Tahlili_N400.xlsx
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jami anketa: 698 | Tahlil: 400 | Sana: 09.09.2026</t>
+          <t>Jami anketa: 698 | Tahlil: 400 | Sana: 18.09.2026</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ish joyida yuqori harorat 47.5% va yuqori shovqin 50.2% deklaratsiya qilingan. 43.2% xodim tez-tez jismoniy charchoq, 31.8% asabiylashish belgilaydi. Bu omillar EnergoHealth-Predict tizimida kelajakdagi kasallanish xavfini oshiruvchi signallar sifatida hisobga olinadi.</t>
+          <t>Ish joyida yuqori harorat 47.5% va yuqori shovqin 50.2% deklaratsiya qilingan. 43.2% xodim tez-tez jismoniy charchoq, 31.8% asabiylashish belgilaydi. Bu omillar Noinfeksion kardiologik xavflarni prognozlash va monitoring qilish milliy-ilmiy ko'p rolli portali tizimida kelajakdagi kasallanish xavfini oshiruvchi signallar sifatida hisobga olinadi.</t>
         </is>
       </c>
     </row>
@@ -538,12 +538,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Xavf prognozi (EnergoHealth-Predict)</t>
+          <t>Xavf prognozi (Noinfeksion kardiologik xavflarni prognozlash va monitoring qilish milliy-ilmiy ko'p rolli portali)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EnergoHealth-Predict tizimi 75 savollik anketa asosida har bir xodim uchun kasallanish xavfini erta baholaydi. 400 nafar namunada o'rtacha xavf balli 57.4%. Yashil zona (past xavf): 35 nafar (8.8%) — kelajakda kasallanish ehtimoli past. Sariq zona (o'rtacha): 334 nafar (83.5%) — profilaktik nazorat talab etiladi. Qizil zona (yuqori): 31 nafar (7.8%) — tezkor tibbiy ko'rik va intervensiya zarur. Tizim klinik tashxis o'rnini bosmaydi, faqat xavfni erta aniqlash uchun mo'ljallangan.</t>
+          <t>Noinfeksion kardiologik xavflarni prognozlash va monitoring qilish milliy-ilmiy ko'p rolli portali tizimi 75 savollik anketa asosida har bir xodim uchun kasallanish xavfini erta baholaydi. 400 nafar namunada o'rtacha xavf balli 57.4%. Yashil zona (past xavf): 35 nafar (8.8%) — kelajakda kasallanish ehtimoli past. Sariq zona (o'rtacha): 334 nafar (83.5%) — profilaktik nazorat talab etiladi. Qizil zona (yuqori): 31 nafar (7.8%) — tezkor tibbiy ko'rik va intervensiya zarur. Tizim klinik tashxis o'rnini bosmaydi, faqat xavfni erta aniqlash uchun mo'ljallangan.</t>
         </is>
       </c>
     </row>
@@ -17019,7 +17019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17045,6 +17045,11 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>95% CI</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Ma'nosi</t>
         </is>
       </c>
@@ -17068,6 +17073,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>6.0–11.5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Past xavf (yashil, &lt;35%) — kelajakda kasallanish ehtimoli nisbatan past</t>
         </is>
       </c>
@@ -17091,6 +17101,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>79.9–87.1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>O'rtacha xavf (sariq, 35–69%) — profilaktik nazorat talab etiladi</t>
         </is>
       </c>
@@ -17113,6 +17128,11 @@
         <v>7.8</v>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>5.1–10.4</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Yuqori xavf (qizil, ≥70%) — tezkor tibbiy ko'rik va profilaktika zarur</t>
         </is>
@@ -17139,7 +17159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17163,6 +17183,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -17181,6 +17206,11 @@
       <c r="D2" t="n">
         <v>82</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>78.2–85.8</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17199,6 +17229,11 @@
       <c r="D3" t="n">
         <v>18</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>14.2–21.8</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17217,6 +17252,11 @@
       <c r="D4" t="n">
         <v>78</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>73.9–82.1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17235,6 +17275,11 @@
       <c r="D5" t="n">
         <v>14</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>10.6–17.4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17253,6 +17298,11 @@
       <c r="D6" t="n">
         <v>12</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>8.8–15.2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17271,6 +17321,11 @@
       <c r="D7" t="n">
         <v>88</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>84.8–91.2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17289,6 +17344,11 @@
       <c r="D8" t="n">
         <v>22</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>17.9–26.1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17307,6 +17367,11 @@
       <c r="D9" t="n">
         <v>18</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>14.2–21.8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17325,6 +17390,11 @@
       <c r="D10" t="n">
         <v>28</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>23.6–32.4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17343,6 +17413,11 @@
       <c r="D11" t="n">
         <v>20</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>16.1–23.9</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17361,6 +17436,11 @@
       <c r="D12" t="n">
         <v>30</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>25.5–34.5</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17379,6 +17459,11 @@
       <c r="D13" t="n">
         <v>50</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>45.1–54.9</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17397,6 +17482,11 @@
       <c r="D14" t="n">
         <v>71</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>66.6–75.4</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17414,6 +17504,11 @@
       </c>
       <c r="D15" t="n">
         <v>29</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>24.6–33.4</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -17427,7 +17522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17451,6 +17546,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -17469,6 +17569,11 @@
       <c r="D2" t="n">
         <v>50.2</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>45.4–55.1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17487,6 +17592,11 @@
       <c r="D3" t="n">
         <v>49.8</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>44.9–54.6</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17505,6 +17615,11 @@
       <c r="D4" t="n">
         <v>47.5</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>42.6–52.4</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17523,6 +17638,11 @@
       <c r="D5" t="n">
         <v>58.5</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>53.7–63.3</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17541,6 +17661,11 @@
       <c r="D6" t="n">
         <v>39.8</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>35.0–44.5</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17559,6 +17684,11 @@
       <c r="D7" t="n">
         <v>37.8</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>33.0–42.5</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17577,6 +17707,11 @@
       <c r="D8" t="n">
         <v>36</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>31.3–40.7</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17595,6 +17730,11 @@
       <c r="D9" t="n">
         <v>56.8</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>51.9–61.6</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17613,6 +17753,11 @@
       <c r="D10" t="n">
         <v>43.2</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>38.4–48.1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17631,6 +17776,11 @@
       <c r="D11" t="n">
         <v>31.8</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>27.2–36.3</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17649,6 +17799,11 @@
       <c r="D12" t="n">
         <v>56.5</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>51.6–61.4</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17667,6 +17822,11 @@
       <c r="D13" t="n">
         <v>34.5</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>29.8–39.2</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17685,6 +17845,11 @@
       <c r="D14" t="n">
         <v>30.5</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>26.0–35.0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17703,6 +17868,11 @@
       <c r="D15" t="n">
         <v>48</v>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>43.1–52.9</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -17720,6 +17890,11 @@
       </c>
       <c r="D16" t="n">
         <v>46</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>41.1–50.9</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -17733,7 +17908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17757,6 +17932,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -17775,6 +17955,11 @@
       <c r="D2" t="n">
         <v>30</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>25.5–34.5</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -17793,6 +17978,11 @@
       <c r="D3" t="n">
         <v>55</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>50.1–59.9</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -17811,6 +18001,11 @@
       <c r="D4" t="n">
         <v>11</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>7.9–14.1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -17829,6 +18024,11 @@
       <c r="D5" t="n">
         <v>55.2</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>50.4–60.1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17847,6 +18047,11 @@
       <c r="D6" t="n">
         <v>63.2</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>58.5–68.0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17865,6 +18070,11 @@
       <c r="D7" t="n">
         <v>20.5</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>16.5–24.5</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17883,6 +18093,11 @@
       <c r="D8" t="n">
         <v>11.8</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>8.6–14.9</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17901,6 +18116,11 @@
       <c r="D9" t="n">
         <v>18</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>14.2–21.8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17919,6 +18139,11 @@
       <c r="D10" t="n">
         <v>30.8</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>26.2–35.3</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17937,6 +18162,11 @@
       <c r="D11" t="n">
         <v>49.5</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>44.6–54.4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17955,6 +18185,11 @@
       <c r="D12" t="n">
         <v>68.8</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>64.2–73.3</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17972,6 +18207,11 @@
       </c>
       <c r="D13" t="n">
         <v>42.2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>37.4–47.1</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -17985,7 +18225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18009,6 +18249,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18027,6 +18272,11 @@
       <c r="D2" t="n">
         <v>21.5</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>17.5–25.5</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18045,6 +18295,11 @@
       <c r="D3" t="n">
         <v>78.5</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>74.5–82.5</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18063,6 +18318,11 @@
       <c r="D4" t="n">
         <v>36.5</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>31.8–41.2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18081,6 +18341,11 @@
       <c r="D5" t="n">
         <v>63.5</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>58.8–68.2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18099,6 +18364,11 @@
       <c r="D6" t="n">
         <v>24</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>19.8–28.2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18116,6 +18386,11 @@
       </c>
       <c r="D7" t="n">
         <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.0–0.0</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -18129,7 +18404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18153,6 +18428,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18171,6 +18451,11 @@
       <c r="D2" t="n">
         <v>73.8</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>69.4–78.1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18189,6 +18474,11 @@
       <c r="D3" t="n">
         <v>24.2</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>20.0–28.5</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18207,6 +18497,11 @@
       <c r="D4" t="n">
         <v>65.2</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>60.6–69.9</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18225,6 +18520,11 @@
       <c r="D5" t="n">
         <v>65</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>60.3–69.7</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18243,6 +18543,11 @@
       <c r="D6" t="n">
         <v>47.8</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>42.9–52.6</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18261,6 +18566,11 @@
       <c r="D7" t="n">
         <v>52.2</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>47.4–57.1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18278,6 +18588,11 @@
       </c>
       <c r="D8" t="n">
         <v>70.2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>65.8–74.7</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -18291,7 +18606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18315,6 +18630,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18333,6 +18653,11 @@
       <c r="D2" t="n">
         <v>49</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>44.1–53.9</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18351,6 +18676,11 @@
       <c r="D3" t="n">
         <v>17</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>13.3–20.7</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18369,6 +18699,11 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.0–0.0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18387,6 +18722,11 @@
       <c r="D5" t="n">
         <v>69</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>64.5–73.5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18405,6 +18745,11 @@
       <c r="D6" t="n">
         <v>71.8</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>67.3–76.2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18423,6 +18768,11 @@
       <c r="D7" t="n">
         <v>43.8</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>38.9–48.6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18441,6 +18791,11 @@
       <c r="D8" t="n">
         <v>49.8</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>44.9–54.6</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18459,6 +18814,11 @@
       <c r="D9" t="n">
         <v>69.2</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>64.7–73.8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -18477,6 +18837,11 @@
       <c r="D10" t="n">
         <v>47</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>42.1–51.9</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -18494,6 +18859,11 @@
       </c>
       <c r="D11" t="n">
         <v>53</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>48.1–57.9</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -18507,7 +18877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18531,6 +18901,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18549,6 +18924,11 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.0–0.0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18567,6 +18947,11 @@
       <c r="D3" t="n">
         <v>34.2</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>29.6–38.9</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18585,6 +18970,11 @@
       <c r="D4" t="n">
         <v>42.5</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>37.7–47.3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18603,6 +18993,11 @@
       <c r="D5" t="n">
         <v>13</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>9.7–16.3</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18620,6 +19015,11 @@
       </c>
       <c r="D6" t="n">
         <v>63.7</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>59.0–68.5</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>